<commit_message>
One pager da #1744 refeito sem Pátio Gourmet e Mari Mari; Pátio Gourmet sai do RD
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-crm-analise-2026-10-15.xlsx
+++ b/docs/nekt/inventario-crm-analise-2026-10-15.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -521,6 +521,18 @@
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Planilha DIVISÃO DE CLIENTE POR SQUAD, aba DIVISÃO DE ANALISTAS MKT DIGITAL (53 linhas, uma repetida). Não traz coluna de HubSpot nem de Google Analytics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Atualização de 16/10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pátio Gourmet saiu do escopo de RD (ex-cliente, informado pela Jussara). Clientes com plano de RD e sem fonte: 20 → 19. O resto do inventário não foi remedido.</t>
         </is>
       </c>
     </row>
@@ -653,22 +665,18 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>SEM FONTE — tem plano de RD na planilha</t>
+          <t>Fora do escopo</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>a levantar</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>a levantar</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Ex-cliente: saiu da agência (informado pela Jussara em 16/10). Sem fonte RD e sem necessidade de criar.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4214,7 +4222,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>RD: 20 clientes com plano de RD na planilha e sem fonte na Nekt</t>
+          <t>RD: 19 clientes com plano de RD na planilha e sem fonte na Nekt (Pátio Gourmet saiu: ex-cliente)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">

</xml_diff>